<commit_message>
zone wise and charts
</commit_message>
<xml_diff>
--- a/output/comparison/comparison.xlsx
+++ b/output/comparison/comparison.xlsx
@@ -462,22 +462,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>57.15</v>
+        <v>70.75</v>
       </c>
       <c r="D2" t="n">
-        <v>69.86</v>
+        <v>82.53</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>91.67</v>
       </c>
       <c r="F2" t="n">
-        <v>53.24</v>
+        <v>35.84</v>
       </c>
       <c r="G2" t="n">
-        <v>13.97</v>
+        <v>46.86</v>
       </c>
     </row>
     <row r="3">
@@ -490,19 +490,19 @@
         <v>22</v>
       </c>
       <c r="C3" t="n">
-        <v>60.51</v>
+        <v>60.59</v>
       </c>
       <c r="D3" t="n">
-        <v>76.36</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>61.36</v>
+        <v>34.5</v>
       </c>
       <c r="G3" t="n">
-        <v>8</v>
+        <v>26.03</v>
       </c>
     </row>
     <row r="4">
@@ -515,19 +515,19 @@
         <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>50.39</v>
+        <v>57.25</v>
       </c>
       <c r="D4" t="n">
-        <v>65.03</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>90</v>
+        <v>91.67</v>
       </c>
       <c r="F4" t="n">
-        <v>45.44</v>
+        <v>41.97</v>
       </c>
       <c r="G4" t="n">
-        <v>6.92</v>
+        <v>40.39</v>
       </c>
     </row>
   </sheetData>
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -589,24 +589,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BJP_amit_shah_puducherry_Ox8IlmYaYnw</t>
+          <t>AIADMK_eps_tirunelveli_uzhdJcMnxTY</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>72.13</v>
+        <v>69.33</v>
       </c>
       <c r="D2" t="n">
-        <v>89.55</v>
+        <v>84.09</v>
       </c>
       <c r="E2" t="n">
-        <v>33.33</v>
+        <v>66.67</v>
       </c>
       <c r="F2" t="n">
-        <v>45.45</v>
+        <v>47.9</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>welfare and funds</t>
+          <t>agriculture and farmers</t>
         </is>
       </c>
     </row>
@@ -618,20 +618,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AIADMK_eps_sivaganga_fHplbO42UOQ</t>
+          <t>BJP_annamalai_unknown_place_eLuZZDLvCG0</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>63.47</v>
+        <v>69.3</v>
       </c>
       <c r="D3" t="n">
-        <v>85.40000000000001</v>
+        <v>86.48999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>55.56</v>
+        <v>58.33</v>
       </c>
       <c r="F3" t="n">
-        <v>65</v>
+        <v>25.4</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -647,24 +647,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BJP_annamalai_unknown_place_w6T-z7DmPvE</t>
+          <t>BJP_annamalai_kangeyam_DoUrt4-ENaI</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>61.9</v>
+        <v>62.93</v>
       </c>
       <c r="D4" t="n">
-        <v>79.95</v>
+        <v>82.26000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>55.56</v>
+        <v>58.33</v>
       </c>
       <c r="F4" t="n">
-        <v>63.16</v>
+        <v>53.74</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>welfare and funds</t>
+          <t>agriculture and farmers</t>
         </is>
       </c>
     </row>
@@ -676,20 +676,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BJP_annamalai_unknown_place_eLuZZDLvCG0</t>
+          <t>AIADMK_eps_tirunelveli_CboJX5ZS7Yc</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>61</v>
+        <v>58.92</v>
       </c>
       <c r="D5" t="n">
-        <v>79.93000000000001</v>
+        <v>78.8</v>
       </c>
       <c r="E5" t="n">
-        <v>44.44</v>
+        <v>66.67</v>
       </c>
       <c r="F5" t="n">
-        <v>56.52</v>
+        <v>21.44</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -705,24 +705,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AIADMK_eps_tirunelveli_MoolcbHo5Cw</t>
+          <t>BJP_annamalai_manamadurai_w6T-z7DmPvE</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>52.83</v>
+        <v>56.6</v>
       </c>
       <c r="D6" t="n">
-        <v>68.06999999999999</v>
+        <v>64.14</v>
       </c>
       <c r="E6" t="n">
-        <v>55.56</v>
+        <v>50</v>
       </c>
       <c r="F6" t="n">
-        <v>63.34</v>
+        <v>37.84</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>law and order</t>
         </is>
       </c>
     </row>
@@ -734,24 +734,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AIADMK_eps_unknown_place_CboJX5ZS7Yc</t>
+          <t>BJP_annamalai_modakurichi_1Qkod1NMMAQ</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>52.76</v>
+        <v>54.68</v>
       </c>
       <c r="D7" t="n">
-        <v>63.19</v>
+        <v>60.98</v>
       </c>
       <c r="E7" t="n">
-        <v>77.78</v>
+        <v>50</v>
       </c>
       <c r="F7" t="n">
-        <v>46.42</v>
+        <v>28.02</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>agriculture and farmers</t>
+          <t>governance</t>
         </is>
       </c>
     </row>
@@ -767,16 +767,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>51.44</v>
+        <v>54.43</v>
       </c>
       <c r="D8" t="n">
-        <v>65.84999999999999</v>
+        <v>58.91</v>
       </c>
       <c r="E8" t="n">
-        <v>55.56</v>
+        <v>58.33</v>
       </c>
       <c r="F8" t="n">
-        <v>43.49</v>
+        <v>42.65</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -792,24 +792,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AIADMK_eps_tenkasi_ahxboKz3Fks</t>
+          <t>AIADMK_eps_unknown_place_L4MaSsW53Dc</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>42.85</v>
+        <v>51.8</v>
       </c>
       <c r="D9" t="n">
-        <v>60.92</v>
+        <v>69.45999999999999</v>
       </c>
       <c r="E9" t="n">
-        <v>11.11</v>
+        <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>40</v>
+        <v>42.64</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>agriculture and farmers</t>
         </is>
       </c>
     </row>
@@ -821,24 +821,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AIADMK_eps_unknown_place_L4MaSsW53Dc</t>
+          <t>AIADMK_eps_sivaganga_fHplbO42UOQ</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>40.18</v>
+        <v>44.15</v>
       </c>
       <c r="D10" t="n">
-        <v>48.93</v>
+        <v>51.32</v>
       </c>
       <c r="E10" t="n">
-        <v>55.56</v>
+        <v>58.33</v>
       </c>
       <c r="F10" t="n">
-        <v>48.48</v>
+        <v>43.15</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>agriculture and farmers</t>
+          <t>law and order</t>
         </is>
       </c>
     </row>
@@ -850,24 +850,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AIADMK_eps_unknown_place_uzhdJcMnxTY</t>
+          <t>AIADMK_eps_tirunelveli_MoolcbHo5Cw</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>39.89</v>
+        <v>43.41</v>
       </c>
       <c r="D11" t="n">
-        <v>59.27</v>
+        <v>51.76</v>
       </c>
       <c r="E11" t="n">
-        <v>55.56</v>
+        <v>50</v>
       </c>
       <c r="F11" t="n">
-        <v>58.54</v>
+        <v>28.32</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>agriculture and farmers</t>
+          <t>law and order</t>
         </is>
       </c>
     </row>
@@ -879,20 +879,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BJP_annamalai_unknown_place_DoUrt4-ENaI</t>
+          <t>AIADMK_eps_tenkasi_ahxboKz3Fks</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>36.5</v>
+        <v>39.89</v>
       </c>
       <c r="D12" t="n">
-        <v>47.76</v>
+        <v>57.88</v>
       </c>
       <c r="E12" t="n">
-        <v>44.44</v>
+        <v>25</v>
       </c>
       <c r="F12" t="n">
-        <v>34.62</v>
+        <v>60.71</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -908,24 +908,24 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BJP_annamalai_unknown_place_1Qkod1NMMAQ</t>
+          <t>AIADMK_eps_chennai_BQ4RLl3plHA</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>35.71</v>
+        <v>22.4</v>
       </c>
       <c r="D13" t="n">
-        <v>49.74</v>
+        <v>28.14</v>
       </c>
       <c r="E13" t="n">
-        <v>44.44</v>
+        <v>33.33</v>
       </c>
       <c r="F13" t="n">
-        <v>49.99</v>
+        <v>11.1</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>infrastructure</t>
+          <t>governance</t>
         </is>
       </c>
     </row>
@@ -937,20 +937,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AIADMK_eps_unknown_place_BQ4RLl3plHA</t>
+          <t>BJP_annamalai_chennai_cwtK_O8ZUpg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>21.43</v>
+        <v>14.75</v>
       </c>
       <c r="D14" t="n">
-        <v>21.91</v>
+        <v>21.1</v>
       </c>
       <c r="E14" t="n">
-        <v>33.33</v>
+        <v>25</v>
       </c>
       <c r="F14" t="n">
-        <v>63.64</v>
+        <v>22.99</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -961,29 +961,29 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AIADMK</t>
+          <t>DMK</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BJP_annamalai_unknown_place_cwtK_O8ZUpg</t>
+          <t>DMK_mk_stalin_cuddalore_aKCrFuJzmy8</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7.15</v>
+        <v>67.05</v>
       </c>
       <c r="D15" t="n">
-        <v>7.19</v>
+        <v>79.64</v>
       </c>
       <c r="E15" t="n">
-        <v>22.22</v>
+        <v>75</v>
       </c>
       <c r="F15" t="n">
-        <v>66.67</v>
+        <v>36.33</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>welfare and funds</t>
         </is>
       </c>
     </row>
@@ -995,20 +995,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_UDMKDkEzH0Q</t>
+          <t>DMK_mk_stalin_unknown_place_chVcUt_21fY</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>77.41</v>
+        <v>61.84</v>
       </c>
       <c r="D16" t="n">
-        <v>91.25</v>
+        <v>84.81</v>
       </c>
       <c r="E16" t="n">
-        <v>88.89</v>
+        <v>50</v>
       </c>
       <c r="F16" t="n">
-        <v>49.43</v>
+        <v>36.85</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1024,24 +1024,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DMK_udhayanidhi_stalin_unknown_place_Y7tlmqhteHg</t>
+          <t>DMK_mk_stalin_tirupattur_pQPa4Pd0ppw</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>71.44</v>
+        <v>57.13</v>
       </c>
       <c r="D17" t="n">
-        <v>92.90000000000001</v>
+        <v>71.51000000000001</v>
       </c>
       <c r="E17" t="n">
-        <v>44.44</v>
+        <v>58.33</v>
       </c>
       <c r="F17" t="n">
-        <v>45.45</v>
+        <v>39.8</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>welfare and funds</t>
+          <t>governance</t>
         </is>
       </c>
     </row>
@@ -1053,24 +1053,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_aKCrFuJzmy8</t>
+          <t>DMK_mk_stalin_virudhunagar_UDMKDkEzH0Q</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>64.73999999999999</v>
+        <v>55.09</v>
       </c>
       <c r="D18" t="n">
-        <v>69.81</v>
+        <v>71.34</v>
       </c>
       <c r="E18" t="n">
-        <v>100</v>
+        <v>66.67</v>
       </c>
       <c r="F18" t="n">
-        <v>68.89</v>
+        <v>35.86</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>women's development</t>
+          <t>welfare and funds</t>
         </is>
       </c>
     </row>
@@ -1082,20 +1082,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_ngRHXOc5lF4</t>
+          <t>DMK_mk_stalin_ramanathapuram_AUpKk_Tp-wc</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>63.82</v>
+        <v>53.79</v>
       </c>
       <c r="D19" t="n">
-        <v>82.93000000000001</v>
+        <v>71.03</v>
       </c>
       <c r="E19" t="n">
-        <v>77.78</v>
+        <v>50</v>
       </c>
       <c r="F19" t="n">
-        <v>61.42</v>
+        <v>20</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1111,20 +1111,20 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_paramakudi_AUpKk_Tp-wc</t>
+          <t>DMK_mk_stalin_maraimalai_nagar_aORoE36baug</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>63.2</v>
+        <v>51.72</v>
       </c>
       <c r="D20" t="n">
-        <v>78</v>
+        <v>70.67</v>
       </c>
       <c r="E20" t="n">
-        <v>66.67</v>
+        <v>50</v>
       </c>
       <c r="F20" t="n">
-        <v>88.23999999999999</v>
+        <v>32</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1140,24 +1140,24 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_TV6zMFPEzkI</t>
+          <t>DMK_mk_stalin_unknown_place_DE0DS3ommsg</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>60.23</v>
+        <v>51.55</v>
       </c>
       <c r="D21" t="n">
-        <v>71.84999999999999</v>
+        <v>61.64</v>
       </c>
       <c r="E21" t="n">
-        <v>77.78</v>
+        <v>50</v>
       </c>
       <c r="F21" t="n">
-        <v>64.28</v>
+        <v>35.95</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>infrastructure</t>
+          <t>governance</t>
         </is>
       </c>
     </row>
@@ -1169,24 +1169,24 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_maraimalai_nagar_aORoE36baug</t>
+          <t>DMK_trichy_trichy_LI-Qjk5zAHA</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>58.33</v>
+        <v>50.98</v>
       </c>
       <c r="D22" t="n">
-        <v>80.81999999999999</v>
+        <v>57.75</v>
       </c>
       <c r="E22" t="n">
-        <v>44.44</v>
+        <v>83.33</v>
       </c>
       <c r="F22" t="n">
-        <v>69.23</v>
+        <v>60.91</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>welfare and funds</t>
+          <t>governance</t>
         </is>
       </c>
     </row>
@@ -1198,20 +1198,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DMK_trichy_siva_unknown_place_LI-Qjk5zAHA</t>
+          <t>DMK_mk_stalin_chennai_TV6zMFPEzkI</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>57.14</v>
+        <v>49.68</v>
       </c>
       <c r="D23" t="n">
-        <v>73.42</v>
+        <v>69.45</v>
       </c>
       <c r="E23" t="n">
         <v>66.67</v>
       </c>
       <c r="F23" t="n">
-        <v>66.67</v>
+        <v>37.71</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1227,24 +1227,24 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_1AFj15bLlJ4</t>
+          <t>DMK_mk_stalin_unknown_place_ngRHXOc5lF4</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>57.13</v>
+        <v>49.65</v>
       </c>
       <c r="D24" t="n">
-        <v>71.91</v>
+        <v>67.06999999999999</v>
       </c>
       <c r="E24" t="n">
-        <v>44.44</v>
+        <v>66.67</v>
       </c>
       <c r="F24" t="n">
-        <v>46.67</v>
+        <v>39.69</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>infrastructure</t>
+          <t>welfare and funds</t>
         </is>
       </c>
     </row>
@@ -1256,24 +1256,24 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_tirupattur_pQPa4Pd0ppw</t>
+          <t>DMK_mk_stalin_paramakudi_iHVeFRPV8DE</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>52.97</v>
+        <v>48.83</v>
       </c>
       <c r="D25" t="n">
-        <v>71.20999999999999</v>
+        <v>71.94</v>
       </c>
       <c r="E25" t="n">
-        <v>55.56</v>
+        <v>58.33</v>
       </c>
       <c r="F25" t="n">
-        <v>75</v>
+        <v>24.85</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>welfare and funds</t>
         </is>
       </c>
     </row>
@@ -1285,24 +1285,24 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_viluppuram_SfLsBzeCaNM</t>
+          <t>DMK_udhayanidhi_stalin_chennai_-n_Pncm6mQo</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>51.2</v>
+        <v>48.08</v>
       </c>
       <c r="D26" t="n">
-        <v>59.34</v>
+        <v>70.06999999999999</v>
       </c>
       <c r="E26" t="n">
-        <v>55.56</v>
+        <v>33.33</v>
       </c>
       <c r="F26" t="n">
-        <v>54.35</v>
+        <v>30.23</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>social justice and deprived communities</t>
+          <t>welfare and funds</t>
         </is>
       </c>
     </row>
@@ -1314,24 +1314,24 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DMK_udhayanidhi_stalin_coimbatore_XkvQRmpEiTA</t>
+          <t>DMK_mk_stalin_unknown_place_W_V1EUi115U</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>49.39</v>
+        <v>46.51</v>
       </c>
       <c r="D27" t="n">
-        <v>66.77</v>
+        <v>60.14</v>
       </c>
       <c r="E27" t="n">
-        <v>33.33</v>
+        <v>58.33</v>
       </c>
       <c r="F27" t="n">
-        <v>33.34</v>
+        <v>33.78</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>infrastructure</t>
+          <t>welfare and funds</t>
         </is>
       </c>
     </row>
@@ -1343,24 +1343,24 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_paramakudi_iHVeFRPV8DE</t>
+          <t>DMK_mk_stalin_unknown_place_01ZulxQ8Ffo</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>46.91</v>
+        <v>45.86</v>
       </c>
       <c r="D28" t="n">
-        <v>52.16</v>
+        <v>37.06</v>
       </c>
       <c r="E28" t="n">
-        <v>77.78</v>
+        <v>91.67</v>
       </c>
       <c r="F28" t="n">
-        <v>75.86</v>
+        <v>34.95</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>infrastructure</t>
+          <t>women's development</t>
         </is>
       </c>
     </row>
@@ -1372,24 +1372,24 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DMK_udhayanidhi_stalin_unknown_place_-n_Pncm6mQo</t>
+          <t>DMK_mk_stalin_cuddalore_SfLsBzeCaNM</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>46.75</v>
+        <v>42.63</v>
       </c>
       <c r="D29" t="n">
-        <v>63.96</v>
+        <v>52.77</v>
       </c>
       <c r="E29" t="n">
-        <v>44.44</v>
+        <v>50</v>
       </c>
       <c r="F29" t="n">
-        <v>73.33</v>
+        <v>29.07</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>education</t>
+          <t>governance</t>
         </is>
       </c>
     </row>
@@ -1401,24 +1401,24 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_01ZulxQ8Ffo</t>
+          <t>DMK_udhayanidhi_stalin_unknown_place_Y7tlmqhteHg</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>46.16</v>
+        <v>42.27</v>
       </c>
       <c r="D30" t="n">
-        <v>42.91</v>
+        <v>64.77</v>
       </c>
       <c r="E30" t="n">
-        <v>88.89</v>
+        <v>33.33</v>
       </c>
       <c r="F30" t="n">
-        <v>71.88</v>
+        <v>24.19</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>women's development</t>
+          <t>welfare and funds</t>
         </is>
       </c>
     </row>
@@ -1430,24 +1430,24 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_DE0DS3ommsg</t>
+          <t>DMK_mk_stalin_unknown_place_d56lS5zIsg0</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>41.66</v>
+        <v>38.67</v>
       </c>
       <c r="D31" t="n">
-        <v>46.36</v>
+        <v>49.28</v>
       </c>
       <c r="E31" t="n">
-        <v>66.67</v>
+        <v>33.33</v>
       </c>
       <c r="F31" t="n">
-        <v>80</v>
+        <v>43.59</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>religion and culture</t>
         </is>
       </c>
     </row>
@@ -1459,24 +1459,24 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DMK_udhayanidhi_stalin_unknown_place_TDzlhqG14Js</t>
+          <t>DMK_udhayanidhi_stalin_coimbatore_XkvQRmpEiTA</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>39.28</v>
+        <v>37.81</v>
       </c>
       <c r="D32" t="n">
-        <v>56.85</v>
+        <v>48.33</v>
       </c>
       <c r="E32" t="n">
-        <v>33.33</v>
+        <v>25</v>
       </c>
       <c r="F32" t="n">
-        <v>50</v>
+        <v>31.63</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>infrastructure</t>
+          <t>governance</t>
         </is>
       </c>
     </row>
@@ -1488,20 +1488,20 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_chVcUt_21fY</t>
+          <t>DMK_mk_stalin_unknown_place_1AFj15bLlJ4</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>35.7</v>
+        <v>37.66</v>
       </c>
       <c r="D33" t="n">
-        <v>46.06</v>
+        <v>59.51</v>
       </c>
       <c r="E33" t="n">
-        <v>55.56</v>
+        <v>33.33</v>
       </c>
       <c r="F33" t="n">
-        <v>61.54</v>
+        <v>48.84</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1517,24 +1517,24 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_W_V1EUi115U</t>
+          <t>DMK_udhayanidhi_stalin_unknown_place_TDzlhqG14Js</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>32.29</v>
+        <v>33.6</v>
       </c>
       <c r="D34" t="n">
-        <v>27.84</v>
+        <v>56.91</v>
       </c>
       <c r="E34" t="n">
-        <v>55.56</v>
+        <v>25</v>
       </c>
       <c r="F34" t="n">
-        <v>84.62</v>
+        <v>30.43</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>infrastructure</t>
+          <t>welfare and funds</t>
         </is>
       </c>
     </row>
@@ -1546,20 +1546,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_d56lS5zIsg0</t>
+          <t>DMK_mk_stalin_unknown_place_em3bCByg2nw</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>28.56</v>
+        <v>29.32</v>
       </c>
       <c r="D35" t="n">
-        <v>33.66</v>
+        <v>37.16</v>
       </c>
       <c r="E35" t="n">
-        <v>22.22</v>
+        <v>33.33</v>
       </c>
       <c r="F35" t="n">
-        <v>28.57</v>
+        <v>36</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1575,53 +1575,53 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DMK_mk_stalin_unknown_place_em3bCByg2nw</t>
+          <t>DMK_kanimozhi_thoothukudi_qBXEjDhB4ng</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>12.49</v>
+        <v>21.31</v>
       </c>
       <c r="D36" t="n">
-        <v>12.54</v>
+        <v>35.75</v>
       </c>
       <c r="E36" t="n">
-        <v>33.33</v>
+        <v>25</v>
       </c>
       <c r="F36" t="n">
-        <v>33.34</v>
+        <v>16.31</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>religion and culture</t>
+          <t>governance</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DMK</t>
+          <t>TVK</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DMK_kanimozhi_thoothukudi_qBXEjDhB4ng</t>
+          <t>TVK_vijay_tiruppur_Ou_H8MFscNg</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>10.71</v>
+        <v>56.22</v>
       </c>
       <c r="D37" t="n">
-        <v>15.22</v>
+        <v>79.97</v>
       </c>
       <c r="E37" t="n">
-        <v>22.22</v>
+        <v>50</v>
       </c>
       <c r="F37" t="n">
-        <v>67.8</v>
+        <v>93.22</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>employment and jobs</t>
         </is>
       </c>
     </row>
@@ -1633,20 +1633,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TVK_vijay_kanyakumari_-Wf1hR8HfhY</t>
+          <t>TVK_vijay_unknown_place_gxUKFr63JAo</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>62.67</v>
+        <v>52.6</v>
       </c>
       <c r="D38" t="n">
-        <v>84.66</v>
+        <v>74.48</v>
       </c>
       <c r="E38" t="n">
         <v>50</v>
       </c>
       <c r="F38" t="n">
-        <v>58.44</v>
+        <v>26.6</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1662,24 +1662,24 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TVK_vijay_unknown_place_gxUKFr63JAo</t>
+          <t>TVK_vijay_vellore_tvY9dOx-flc</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>60.27</v>
+        <v>45.59</v>
       </c>
       <c r="D39" t="n">
-        <v>83.63</v>
+        <v>52.4</v>
       </c>
       <c r="E39" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F39" t="n">
-        <v>60.64</v>
+        <v>36.27</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>welfare and funds</t>
+          <t>governance</t>
         </is>
       </c>
     </row>
@@ -1691,20 +1691,20 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TVK_vijay_puducherry_66uCCl2jD_s</t>
+          <t>TVK_vijay_kanyakumari_-Wf1hR8HfhY</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>47.64</v>
+        <v>44.31</v>
       </c>
       <c r="D40" t="n">
-        <v>61.04</v>
+        <v>63.4</v>
       </c>
       <c r="E40" t="n">
-        <v>40</v>
+        <v>41.67</v>
       </c>
       <c r="F40" t="n">
-        <v>64.70999999999999</v>
+        <v>88.77</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1720,24 +1720,24 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TVK_vijay_tiruppur_Ou_H8MFscNg</t>
+          <t>TVK_vijay_chennai_F3qWCkrErcs</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>44.67</v>
+        <v>39.69</v>
       </c>
       <c r="D41" t="n">
-        <v>73.37</v>
+        <v>55.43</v>
       </c>
       <c r="E41" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F41" t="n">
-        <v>75</v>
+        <v>31.03</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>welfare and funds</t>
+          <t>governance</t>
         </is>
       </c>
     </row>
@@ -1749,24 +1749,24 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TVK_vijay_vellore_tvY9dOx-flc</t>
+          <t>TVK_vijay_puducherry_66uCCl2jD_s</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>43.08</v>
+        <v>39.22</v>
       </c>
       <c r="D42" t="n">
-        <v>53.29</v>
+        <v>57.43</v>
       </c>
       <c r="E42" t="n">
-        <v>50</v>
+        <v>33.33</v>
       </c>
       <c r="F42" t="n">
-        <v>44.83</v>
+        <v>33.19</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>welfare and funds</t>
         </is>
       </c>
     </row>
@@ -1778,20 +1778,20 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TVK_vijay_karur_-W7wFFgwVuw</t>
+          <t>TVK_vijay_unknown_place_AycUJ5Ygo-E</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>36.71</v>
+        <v>39.22</v>
       </c>
       <c r="D43" t="n">
-        <v>41.74</v>
+        <v>53.84</v>
       </c>
       <c r="E43" t="n">
-        <v>40</v>
+        <v>66.67</v>
       </c>
       <c r="F43" t="n">
-        <v>46.67</v>
+        <v>41.2</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1807,20 +1807,20 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>TVK_vijay_unknown_place_AycUJ5Ygo-E</t>
+          <t>TVK_vijay_unknown_place_El6qxC-DR48</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>36.53</v>
+        <v>35.07</v>
       </c>
       <c r="D44" t="n">
-        <v>44.38</v>
+        <v>53.79</v>
       </c>
       <c r="E44" t="n">
-        <v>70</v>
+        <v>33.33</v>
       </c>
       <c r="F44" t="n">
-        <v>43.86</v>
+        <v>24.46</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1836,20 +1836,20 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>TVK_vijay_chennai_F3qWCkrErcs</t>
+          <t>TVK_vijay_unknown_place_QHdUI8CBqq8</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>31.1</v>
+        <v>35.07</v>
       </c>
       <c r="D45" t="n">
-        <v>44.85</v>
+        <v>52.29</v>
       </c>
       <c r="E45" t="n">
-        <v>50</v>
+        <v>33.33</v>
       </c>
       <c r="F45" t="n">
-        <v>44.09</v>
+        <v>31.34</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1869,16 +1869,16 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>26.66</v>
+        <v>34.76</v>
       </c>
       <c r="D46" t="n">
-        <v>34.22</v>
+        <v>45.51</v>
       </c>
       <c r="E46" t="n">
-        <v>40</v>
+        <v>58.33</v>
       </c>
       <c r="F46" t="n">
-        <v>29.4</v>
+        <v>20.22</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1894,20 +1894,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>TVK_vijay_unknown_place_QHdUI8CBqq8</t>
+          <t>TVK_vijay_tirunelveli_jx93xjr4Z50</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>25.12</v>
+        <v>33.66</v>
       </c>
       <c r="D47" t="n">
-        <v>41.67</v>
+        <v>48.88</v>
       </c>
       <c r="E47" t="n">
-        <v>30</v>
+        <v>33.33</v>
       </c>
       <c r="F47" t="n">
-        <v>50</v>
+        <v>34.77</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1923,24 +1923,24 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TVK_vijay_tirunelveli_jx93xjr4Z50</t>
+          <t>TVK_vijay_karur_-W7wFFgwVuw</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>23.09</v>
+        <v>22.46</v>
       </c>
       <c r="D48" t="n">
-        <v>39.64</v>
+        <v>19.71</v>
       </c>
       <c r="E48" t="n">
-        <v>30</v>
+        <v>41.67</v>
       </c>
       <c r="F48" t="n">
-        <v>57.9</v>
+        <v>68.47</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>health</t>
         </is>
       </c>
     </row>
@@ -1952,24 +1952,24 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TVK_vijay_unknown_place_El6qxC-DR48</t>
+          <t>TVK_vijay_unknown_place_eqSUQwp3l14</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>14</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="D49" t="n">
-        <v>31.89</v>
+        <v>16.25</v>
       </c>
       <c r="E49" t="n">
-        <v>20</v>
+        <v>16.67</v>
       </c>
       <c r="F49" t="n">
-        <v>56</v>
+        <v>100</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>religion and culture</t>
         </is>
       </c>
     </row>
@@ -2028,35 +2028,6 @@
       <c r="G51" t="inlineStr">
         <is>
           <t>agriculture and farmers</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>TVK</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>TVK_vijay_unknown_place_eqSUQwp3l14</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E52" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" t="n">
-        <v>50</v>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>religion and culture</t>
         </is>
       </c>
     </row>
@@ -2113,13 +2084,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3.58</v>
+        <v>19.68</v>
       </c>
       <c r="D2" t="n">
-        <v>10.07</v>
+        <v>21</v>
       </c>
       <c r="E2" t="n">
-        <v>6.49</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="3">
@@ -2134,13 +2105,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>2.73</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>-2.73</v>
       </c>
     </row>
     <row r="4">
@@ -2155,13 +2126,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7.14</v>
+        <v>1.1</v>
       </c>
       <c r="D4" t="n">
-        <v>1.55</v>
+        <v>2.72</v>
       </c>
       <c r="E4" t="n">
-        <v>-5.59</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="5">
@@ -2176,13 +2147,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>17.85</v>
+        <v>16.39</v>
       </c>
       <c r="D5" t="n">
-        <v>7.35</v>
+        <v>3.96</v>
       </c>
       <c r="E5" t="n">
-        <v>-10.5</v>
+        <v>-12.42</v>
       </c>
     </row>
     <row r="6">
@@ -2197,13 +2168,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>5.46</v>
       </c>
       <c r="D6" t="n">
-        <v>23.38</v>
+        <v>19.53</v>
       </c>
       <c r="E6" t="n">
-        <v>23.38</v>
+        <v>14.07</v>
       </c>
     </row>
     <row r="7">
@@ -2218,13 +2189,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3.58</v>
+        <v>3.28</v>
       </c>
       <c r="D7" t="n">
-        <v>4.02</v>
+        <v>1.12</v>
       </c>
       <c r="E7" t="n">
-        <v>0.44</v>
+        <v>-2.15</v>
       </c>
     </row>
     <row r="8">
@@ -2239,13 +2210,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>14.28</v>
+        <v>10.39</v>
       </c>
       <c r="D8" t="n">
-        <v>11.75</v>
+        <v>6.7</v>
       </c>
       <c r="E8" t="n">
-        <v>-2.53</v>
+        <v>-3.69</v>
       </c>
     </row>
     <row r="9">
@@ -2260,13 +2231,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3.58</v>
+        <v>3.28</v>
       </c>
       <c r="D9" t="n">
-        <v>14.78</v>
+        <v>15.52</v>
       </c>
       <c r="E9" t="n">
-        <v>11.21</v>
+        <v>12.24</v>
       </c>
     </row>
     <row r="10">
@@ -2281,13 +2252,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>2.73</v>
       </c>
       <c r="D10" t="n">
-        <v>1.33</v>
+        <v>1.74</v>
       </c>
       <c r="E10" t="n">
-        <v>1.33</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="11">
@@ -2302,13 +2273,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3.58</v>
+        <v>0.54</v>
       </c>
       <c r="D11" t="n">
-        <v>1.65</v>
+        <v>0.47</v>
       </c>
       <c r="E11" t="n">
-        <v>-1.93</v>
+        <v>-0.07000000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -2323,13 +2294,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>42.85</v>
+        <v>28.41</v>
       </c>
       <c r="D12" t="n">
-        <v>22.34</v>
+        <v>21.68</v>
       </c>
       <c r="E12" t="n">
-        <v>-20.51</v>
+        <v>-6.73</v>
       </c>
     </row>
     <row r="13">
@@ -2344,13 +2315,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3.58</v>
+        <v>6.01</v>
       </c>
       <c r="D13" t="n">
-        <v>1.79</v>
+        <v>5.56</v>
       </c>
       <c r="E13" t="n">
-        <v>-1.79</v>
+        <v>-0.45</v>
       </c>
     </row>
     <row r="14">
@@ -2365,13 +2336,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12.5</v>
+        <v>10.11</v>
       </c>
       <c r="D14" t="n">
-        <v>3.04</v>
+        <v>1.8</v>
       </c>
       <c r="E14" t="n">
-        <v>-9.460000000000001</v>
+        <v>-8.31</v>
       </c>
     </row>
     <row r="15">
@@ -2386,13 +2357,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1.37</v>
       </c>
       <c r="D15" t="n">
         <v>0.39</v>
       </c>
       <c r="E15" t="n">
-        <v>0.39</v>
+        <v>-0.98</v>
       </c>
     </row>
     <row r="16">
@@ -2407,13 +2378,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>12.5</v>
+        <v>8.75</v>
       </c>
       <c r="D16" t="n">
-        <v>6.36</v>
+        <v>2.63</v>
       </c>
       <c r="E16" t="n">
-        <v>-6.14</v>
+        <v>-6.12</v>
       </c>
     </row>
     <row r="17">
@@ -2428,13 +2399,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.71</v>
+        <v>19.4</v>
       </c>
       <c r="D17" t="n">
-        <v>3.79</v>
+        <v>3.82</v>
       </c>
       <c r="E17" t="n">
-        <v>-6.92</v>
+        <v>-15.58</v>
       </c>
     </row>
     <row r="18">
@@ -2449,13 +2420,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5.36</v>
+        <v>10.38</v>
       </c>
       <c r="D18" t="n">
-        <v>17.52</v>
+        <v>26.4</v>
       </c>
       <c r="E18" t="n">
-        <v>12.16</v>
+        <v>16.02</v>
       </c>
     </row>
     <row r="19">
@@ -2470,13 +2441,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>2.74</v>
       </c>
       <c r="D19" t="n">
-        <v>1.99</v>
+        <v>0.61</v>
       </c>
       <c r="E19" t="n">
-        <v>1.99</v>
+        <v>-2.13</v>
       </c>
     </row>
     <row r="20">
@@ -2491,13 +2462,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>10.71</v>
+        <v>11.2</v>
       </c>
       <c r="D20" t="n">
-        <v>23.04</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="E20" t="n">
-        <v>12.33</v>
+        <v>-2.49</v>
       </c>
     </row>
     <row r="21">
@@ -2512,13 +2483,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>1.37</v>
       </c>
       <c r="D21" t="n">
-        <v>1.79</v>
+        <v>0.54</v>
       </c>
       <c r="E21" t="n">
-        <v>1.79</v>
+        <v>-0.83</v>
       </c>
     </row>
     <row r="22">
@@ -2533,13 +2504,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3.57</v>
+        <v>6.01</v>
       </c>
       <c r="D22" t="n">
-        <v>5.75</v>
+        <v>7.54</v>
       </c>
       <c r="E22" t="n">
-        <v>2.18</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="23">
@@ -2554,13 +2525,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5.36</v>
+        <v>6.28</v>
       </c>
       <c r="D23" t="n">
-        <v>4.49</v>
+        <v>3.3</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.87</v>
+        <v>-2.99</v>
       </c>
     </row>
     <row r="24">
@@ -2575,13 +2546,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>35.73</v>
+        <v>17.76</v>
       </c>
       <c r="D24" t="n">
-        <v>19.63</v>
+        <v>34.16</v>
       </c>
       <c r="E24" t="n">
-        <v>-16.1</v>
+        <v>16.41</v>
       </c>
     </row>
     <row r="25">
@@ -2596,13 +2567,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3.57</v>
+        <v>4.64</v>
       </c>
       <c r="D25" t="n">
-        <v>12.21</v>
+        <v>10.09</v>
       </c>
       <c r="E25" t="n">
-        <v>8.65</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="26">
@@ -2617,13 +2588,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>12</v>
+        <v>11.08</v>
       </c>
       <c r="D26" t="n">
-        <v>3.83</v>
+        <v>4.5</v>
       </c>
       <c r="E26" t="n">
-        <v>-8.17</v>
+        <v>-6.57</v>
       </c>
     </row>
     <row r="27">
@@ -2638,13 +2609,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>0.61</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>-4</v>
+        <v>-0.61</v>
       </c>
     </row>
     <row r="28">
@@ -2659,13 +2630,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>8</v>
+        <v>4.31</v>
       </c>
       <c r="D28" t="n">
-        <v>0.85</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E28" t="n">
-        <v>-7.15</v>
+        <v>-3.37</v>
       </c>
     </row>
     <row r="29">
@@ -2680,13 +2651,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>12</v>
+        <v>24.92</v>
       </c>
       <c r="D29" t="n">
-        <v>6.15</v>
+        <v>7.61</v>
       </c>
       <c r="E29" t="n">
-        <v>-5.85</v>
+        <v>-17.32</v>
       </c>
     </row>
     <row r="30">
@@ -2701,13 +2672,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>12</v>
+        <v>15.7</v>
       </c>
       <c r="D30" t="n">
-        <v>40.27</v>
+        <v>31.98</v>
       </c>
       <c r="E30" t="n">
-        <v>28.27</v>
+        <v>16.29</v>
       </c>
     </row>
     <row r="31">
@@ -2722,13 +2693,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>3.08</v>
       </c>
       <c r="D31" t="n">
-        <v>2.2</v>
+        <v>6.44</v>
       </c>
       <c r="E31" t="n">
-        <v>2.2</v>
+        <v>3.36</v>
       </c>
     </row>
     <row r="32">
@@ -2743,13 +2714,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>16</v>
+        <v>13.23</v>
       </c>
       <c r="D32" t="n">
-        <v>3.35</v>
+        <v>1.12</v>
       </c>
       <c r="E32" t="n">
-        <v>-12.65</v>
+        <v>-12.11</v>
       </c>
     </row>
     <row r="33">
@@ -2764,13 +2735,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>1.84</v>
       </c>
       <c r="D33" t="n">
-        <v>8.73</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="E33" t="n">
-        <v>6.73</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="34">
@@ -2785,13 +2756,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>4.62</v>
       </c>
       <c r="D34" t="n">
-        <v>12.4</v>
+        <v>12.03</v>
       </c>
       <c r="E34" t="n">
-        <v>12.4</v>
+        <v>7.41</v>
       </c>
     </row>
     <row r="35">
@@ -2806,13 +2777,13 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>5.99</v>
+        <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>1.47</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="E35" t="n">
-        <v>-4.53</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="36">
@@ -2827,13 +2798,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>24</v>
+        <v>12.92</v>
       </c>
       <c r="D36" t="n">
-        <v>20.02</v>
+        <v>17.61</v>
       </c>
       <c r="E36" t="n">
-        <v>-3.98</v>
+        <v>4.69</v>
       </c>
     </row>
     <row r="37">
@@ -2848,13 +2819,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>3.69</v>
       </c>
       <c r="D37" t="n">
-        <v>0.72</v>
+        <v>0.93</v>
       </c>
       <c r="E37" t="n">
-        <v>-3.28</v>
+        <v>-2.76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>